<commit_message>
Update Konfigurasi.xlsx and add new RAB 2026.xlsx file for project documentation
</commit_message>
<xml_diff>
--- a/Dokumentasi/Konfigurasi.xlsx
+++ b/Dokumentasi/Konfigurasi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pengujian\Ship_Model_Control_ESP32-S3 v2026.01\Dokumentasi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0CED2AF-6BD7-4ACD-BA34-583D97AB4AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D9F9BA6-D158-4427-A863-BE415CBC58E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SN_MacAdress" sheetId="1" r:id="rId1"/>
@@ -887,7 +887,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -924,6 +924,7 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -954,10 +955,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -12971,10 +12968,10 @@
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="14" t="s">
         <v>243</v>
       </c>
     </row>
@@ -13089,7 +13086,7 @@
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="24" t="s">
         <v>220</v>
       </c>
       <c r="C7">
@@ -13108,7 +13105,7 @@
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="23"/>
+      <c r="B8" s="24"/>
       <c r="C8">
         <v>-40</v>
       </c>
@@ -13125,7 +13122,7 @@
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="24" t="s">
         <v>221</v>
       </c>
       <c r="C9">
@@ -13144,7 +13141,7 @@
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="23"/>
+      <c r="B10" s="24"/>
       <c r="C10">
         <v>-35</v>
       </c>
@@ -13161,7 +13158,7 @@
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="24" t="s">
         <v>222</v>
       </c>
       <c r="C11">
@@ -13180,7 +13177,7 @@
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="23"/>
+      <c r="B12" s="24"/>
       <c r="C12">
         <v>-10</v>
       </c>
@@ -13238,7 +13235,7 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="24" t="s">
         <v>220</v>
       </c>
       <c r="C18">
@@ -13257,7 +13254,7 @@
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="23"/>
+      <c r="B19" s="24"/>
       <c r="C19">
         <v>-40</v>
       </c>
@@ -13274,7 +13271,7 @@
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="24" t="s">
         <v>221</v>
       </c>
       <c r="C20">
@@ -13293,7 +13290,7 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="23"/>
+      <c r="B21" s="24"/>
       <c r="C21">
         <v>-35</v>
       </c>
@@ -13310,7 +13307,7 @@
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="24" t="s">
         <v>222</v>
       </c>
       <c r="C22">
@@ -13329,7 +13326,7 @@
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="23"/>
+      <c r="B23" s="24"/>
       <c r="C23">
         <v>-10</v>
       </c>
@@ -13365,11 +13362,11 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
     </row>
     <row r="3" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
@@ -14316,15 +14313,15 @@
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B35" s="14" t="s">
+      <c r="B35" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
@@ -14547,10 +14544,10 @@
       <c r="H45" s="11"/>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B47" s="15" t="s">
+      <c r="B47" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="C47" s="15"/>
+      <c r="C47" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -14601,11 +14598,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>229</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -14850,10 +14847,10 @@
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="B25" s="16"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="3">
         <f>SUM(C4:C24)</f>
         <v>32</v>
@@ -14898,7 +14895,7 @@
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="18" t="s">
         <v>39</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -14915,7 +14912,7 @@
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="17"/>
+      <c r="B5" s="18"/>
       <c r="C5" s="2" t="s">
         <v>37</v>
       </c>
@@ -14930,7 +14927,7 @@
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="17"/>
+      <c r="B6" s="18"/>
       <c r="C6" s="2" t="s">
         <v>38</v>
       </c>
@@ -14945,7 +14942,7 @@
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="17"/>
+      <c r="B7" s="18"/>
       <c r="C7" s="2" t="s">
         <v>41</v>
       </c>
@@ -14960,7 +14957,7 @@
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="18" t="s">
         <v>44</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -14975,7 +14972,7 @@
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="17"/>
+      <c r="B9" s="18"/>
       <c r="C9" s="2" t="s">
         <v>40</v>
       </c>
@@ -14990,7 +14987,7 @@
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="17"/>
+      <c r="B10" s="18"/>
       <c r="C10" s="2" t="s">
         <v>46</v>
       </c>
@@ -15005,7 +15002,7 @@
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="17"/>
+      <c r="B11" s="18"/>
       <c r="C11" s="2" t="s">
         <v>47</v>
       </c>
@@ -15015,12 +15012,12 @@
       <c r="E11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="19" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="17"/>
+      <c r="B12" s="18"/>
       <c r="C12" s="2" t="s">
         <v>48</v>
       </c>
@@ -15030,10 +15027,10 @@
       <c r="E12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="19"/>
+      <c r="F12" s="20"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>51</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -15045,12 +15042,12 @@
       <c r="E13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="18" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="17"/>
+      <c r="B14" s="18"/>
       <c r="C14" s="2" t="s">
         <v>53</v>
       </c>
@@ -15060,10 +15057,10 @@
       <c r="E14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F14" s="17"/>
+      <c r="F14" s="18"/>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="17"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="2" t="s">
         <v>40</v>
       </c>
@@ -15078,7 +15075,7 @@
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="17"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="2" t="s">
         <v>46</v>
       </c>
@@ -15093,7 +15090,7 @@
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="19" t="s">
         <v>108</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -15110,7 +15107,7 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="20"/>
+      <c r="B18" s="21"/>
       <c r="C18" s="2" t="s">
         <v>66</v>
       </c>
@@ -15125,7 +15122,7 @@
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="20"/>
+      <c r="B19" s="21"/>
       <c r="C19" s="2" t="s">
         <v>40</v>
       </c>
@@ -15140,14 +15137,14 @@
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="20"/>
+      <c r="B20" s="21"/>
       <c r="C20" s="2" t="s">
         <v>96</v>
       </c>
       <c r="D20" s="3">
         <v>9</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="19" t="s">
         <v>98</v>
       </c>
       <c r="F20" s="3" t="s">
@@ -15155,20 +15152,20 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="19"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="2" t="s">
         <v>97</v>
       </c>
       <c r="D21" s="3">
         <v>10</v>
       </c>
-      <c r="E21" s="19"/>
+      <c r="E21" s="20"/>
       <c r="F21" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="18" t="s">
         <v>90</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -15180,12 +15177,12 @@
       <c r="E22" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="18" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="17"/>
+      <c r="B23" s="18"/>
       <c r="C23" s="2" t="s">
         <v>53</v>
       </c>
@@ -15195,10 +15192,10 @@
       <c r="E23" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F23" s="17"/>
+      <c r="F23" s="18"/>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="17"/>
+      <c r="B24" s="18"/>
       <c r="C24" s="2" t="s">
         <v>40</v>
       </c>
@@ -15213,7 +15210,7 @@
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="17"/>
+      <c r="B25" s="18"/>
       <c r="C25" s="2" t="s">
         <v>46</v>
       </c>
@@ -15228,7 +15225,7 @@
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="18" t="s">
         <v>105</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -15245,7 +15242,7 @@
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="17"/>
+      <c r="B27" s="18"/>
       <c r="C27" s="2" t="s">
         <v>107</v>
       </c>
@@ -15306,7 +15303,7 @@
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="18" t="s">
         <v>57</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -15314,37 +15311,37 @@
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="17"/>
+      <c r="B4" s="18"/>
       <c r="C4" s="2" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B5" s="17"/>
+      <c r="B5" s="18"/>
       <c r="C5" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B6" s="17"/>
+      <c r="B6" s="18"/>
       <c r="C6" s="2" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B7" s="17"/>
+      <c r="B7" s="18"/>
       <c r="C7" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="17"/>
+      <c r="B8" s="18"/>
       <c r="C8" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B9" s="17"/>
+      <c r="B9" s="18"/>
       <c r="C9" s="2" t="s">
         <v>64</v>
       </c>
@@ -15425,28 +15422,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21" t="s">
+      <c r="C3" s="22"/>
+      <c r="D3" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="21"/>
+      <c r="E3" s="22"/>
       <c r="F3" s="1" t="s">
         <v>33</v>
       </c>
@@ -15980,28 +15977,28 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21" t="s">
+      <c r="C22" s="22"/>
+      <c r="D22" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E22" s="21"/>
+      <c r="E22" s="22"/>
       <c r="F22" s="1" t="s">
         <v>33</v>
       </c>
@@ -16560,11 +16557,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
@@ -17070,7 +17067,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="23" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -17081,7 +17078,7 @@
       </c>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B2" s="22"/>
+      <c r="B2" s="23"/>
       <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
@@ -17090,7 +17087,7 @@
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B3" s="22"/>
+      <c r="B3" s="23"/>
       <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
@@ -17099,7 +17096,7 @@
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B4" s="22"/>
+      <c r="B4" s="23"/>
       <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
@@ -17108,7 +17105,7 @@
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B5" s="22"/>
+      <c r="B5" s="23"/>
       <c r="C5" s="3" t="s">
         <v>15</v>
       </c>
@@ -17117,48 +17114,48 @@
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="18" t="s">
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="17" t="s">
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="19"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="20"/>
       <c r="F9" s="2" t="s">
         <v>20</v>
       </c>
@@ -17179,7 +17176,7 @@
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B10" s="17"/>
+      <c r="B10" s="18"/>
       <c r="C10" s="3" t="s">
         <v>12</v>
       </c>
@@ -17209,7 +17206,7 @@
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B11" s="17"/>
+      <c r="B11" s="18"/>
       <c r="C11" s="3" t="s">
         <v>13</v>
       </c>
@@ -17239,7 +17236,7 @@
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="17"/>
+      <c r="B12" s="18"/>
       <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
@@ -17269,7 +17266,7 @@
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B13" s="17"/>
+      <c r="B13" s="18"/>
       <c r="C13" s="3" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
Remove temporary Excel file and update main Konfigurasi.xlsx file for improved data management
</commit_message>
<xml_diff>
--- a/Dokumentasi/Konfigurasi.xlsx
+++ b/Dokumentasi/Konfigurasi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pengujian\Ship_Model_Control_ESP32-S3 v2026.01\Dokumentasi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D9F9BA6-D158-4427-A863-BE415CBC58E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550E95D4-8426-42C1-8AE9-2BDC4B546AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SN_MacAdress" sheetId="1" r:id="rId1"/>

</xml_diff>